<commit_message>
can build log and know if the loop don't run
</commit_message>
<xml_diff>
--- a/datasehat.xlsx
+++ b/datasehat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Documents\sehatselenium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8CD937-6DE7-44CD-817A-2209422D71B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52E0EDC7-1D0E-4DCA-8A4E-8BA82CB610AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8604" yWindow="1884" windowWidth="14436" windowHeight="8880" xr2:uid="{204D681D-D5A1-4808-BEE3-E0115C09E5E0}"/>
+    <workbookView xWindow="8604" yWindow="3360" windowWidth="14436" windowHeight="8880" xr2:uid="{204D681D-D5A1-4808-BEE3-E0115C09E5E0}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>nama</t>
   </si>
@@ -106,31 +106,13 @@
     <t>alamat</t>
   </si>
   <si>
-    <t>RONGGUR HALOMOAN LUBIS</t>
-  </si>
-  <si>
-    <t>NURYANDI</t>
-  </si>
-  <si>
-    <t>AHMAD BUKHORI</t>
-  </si>
-  <si>
-    <t>SYAM RAGIL RAHARJO</t>
-  </si>
-  <si>
-    <t>SURYA CAHYA DININGRAT</t>
-  </si>
-  <si>
-    <t>DIAN NOVITA SARI</t>
-  </si>
-  <si>
-    <t>USNIAWATI</t>
-  </si>
-  <si>
-    <t>RINI SUTARTI</t>
-  </si>
-  <si>
-    <t>ZIDNA RAHAYU</t>
+    <t>RIYAN ADRIAN WIBISONO</t>
+  </si>
+  <si>
+    <t>MAKSUDI</t>
+  </si>
+  <si>
+    <t>TIYA SETIYA</t>
   </si>
 </sst>
 </file>
@@ -184,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -276,11 +258,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -312,9 +305,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -323,6 +313,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -669,229 +680,145 @@
       <c r="H1" s="3"/>
     </row>
     <row r="2" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="19">
         <v>110</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="20">
         <v>70</v>
       </c>
-      <c r="D2" s="10">
-        <v>156</v>
-      </c>
-      <c r="E2" s="10">
-        <v>92</v>
-      </c>
-      <c r="F2" s="10">
+      <c r="D2" s="20">
+        <v>160</v>
+      </c>
+      <c r="E2" s="20">
+        <v>62</v>
+      </c>
+      <c r="F2" s="20">
         <v>80</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="20">
         <v>82</v>
       </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="11">
-        <v>130</v>
-      </c>
-      <c r="C3" s="12">
-        <v>90</v>
-      </c>
-      <c r="D3" s="12">
-        <v>156</v>
-      </c>
-      <c r="E3" s="12">
+      <c r="B3" s="21">
+        <v>120</v>
+      </c>
+      <c r="C3" s="22">
+        <v>80</v>
+      </c>
+      <c r="D3" s="22">
+        <v>160</v>
+      </c>
+      <c r="E3" s="22">
+        <v>60</v>
+      </c>
+      <c r="F3" s="22">
+        <v>84</v>
+      </c>
+      <c r="G3" s="22">
+        <v>84</v>
+      </c>
+      <c r="H3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="21">
+        <v>110</v>
+      </c>
+      <c r="C4" s="22">
         <v>70</v>
       </c>
-      <c r="F3" s="12">
+      <c r="D4" s="22">
+        <v>158</v>
+      </c>
+      <c r="E4" s="22">
+        <v>56</v>
+      </c>
+      <c r="F4" s="22">
+        <v>80</v>
+      </c>
+      <c r="G4" s="22">
         <v>86</v>
       </c>
-      <c r="G3" s="12">
-        <v>82</v>
-      </c>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="11">
-        <v>100</v>
-      </c>
-      <c r="C4" s="12">
-        <v>70</v>
-      </c>
-      <c r="D4" s="12">
-        <v>158</v>
-      </c>
-      <c r="E4" s="12">
-        <v>55</v>
-      </c>
-      <c r="F4" s="12">
-        <v>86</v>
-      </c>
-      <c r="G4" s="12">
-        <v>83</v>
-      </c>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="11">
-        <v>100</v>
-      </c>
-      <c r="C5" s="12">
-        <v>60</v>
-      </c>
-      <c r="D5" s="12">
-        <v>157</v>
-      </c>
-      <c r="E5" s="12">
-        <v>81</v>
-      </c>
-      <c r="F5" s="12">
-        <v>82</v>
-      </c>
-      <c r="G5" s="12">
-        <v>84</v>
-      </c>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="11">
-        <v>120</v>
-      </c>
-      <c r="C6" s="12">
-        <v>80</v>
-      </c>
-      <c r="D6" s="12">
-        <v>156</v>
-      </c>
-      <c r="E6" s="12">
-        <v>58</v>
-      </c>
-      <c r="F6" s="12">
-        <v>84</v>
-      </c>
-      <c r="G6" s="12">
-        <v>82</v>
-      </c>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="9">
-        <v>110</v>
-      </c>
-      <c r="C7" s="10">
-        <v>70</v>
-      </c>
-      <c r="D7" s="10">
-        <v>156</v>
-      </c>
-      <c r="E7" s="10">
-        <v>64</v>
-      </c>
-      <c r="F7" s="10">
-        <v>84</v>
-      </c>
-      <c r="G7" s="10">
-        <v>89</v>
-      </c>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="11">
-        <v>140</v>
-      </c>
-      <c r="C8" s="12">
-        <v>90</v>
-      </c>
-      <c r="D8" s="12">
-        <v>154</v>
-      </c>
-      <c r="E8" s="12">
-        <v>67</v>
-      </c>
-      <c r="F8" s="12">
-        <v>80</v>
-      </c>
-      <c r="G8" s="12">
-        <v>75</v>
-      </c>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="11">
-        <v>110</v>
-      </c>
-      <c r="C9" s="12">
-        <v>70</v>
-      </c>
-      <c r="D9" s="12">
-        <v>158</v>
-      </c>
-      <c r="E9" s="12">
-        <v>64</v>
-      </c>
-      <c r="F9" s="12">
-        <v>80</v>
-      </c>
-      <c r="G9" s="12">
-        <v>84</v>
-      </c>
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="11">
-        <v>110</v>
-      </c>
-      <c r="C10" s="12">
-        <v>70</v>
-      </c>
-      <c r="D10" s="12">
-        <v>158</v>
-      </c>
-      <c r="E10" s="12">
-        <v>61</v>
-      </c>
-      <c r="F10" s="12">
-        <v>84</v>
-      </c>
-      <c r="G10" s="12">
-        <v>86</v>
-      </c>
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -905,33 +832,26 @@
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
       <c r="H14" s="4"/>
     </row>
     <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
       <c r="H15" s="4"/>
     </row>
     <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -944,7 +864,7 @@
       <c r="G16" s="12"/>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="12"/>
@@ -952,44 +872,46 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
-    </row>
-    <row r="18" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="16"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-    </row>
-    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-    </row>
-    <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H17" s="18"/>
+    </row>
+    <row r="18" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="18"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+    </row>
+    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+    </row>
+    <row r="22" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="11"/>
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
@@ -998,7 +920,7 @@
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
     </row>
-    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="11"/>
       <c r="B23" s="11"/>
       <c r="C23" s="12"/>
@@ -1007,7 +929,7 @@
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
     </row>
-    <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="11"/>
       <c r="B24" s="11"/>
       <c r="C24" s="12"/>
@@ -1016,7 +938,7 @@
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
     </row>
-    <row r="25" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="12"/>
@@ -1025,7 +947,7 @@
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
     </row>
-    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
       <c r="C26" s="12"/>
@@ -1034,95 +956,95 @@
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-    </row>
-    <row r="29" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-    </row>
-    <row r="30" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="16"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-    </row>
-    <row r="31" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="16"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-    </row>
-    <row r="32" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="16"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+    </row>
+    <row r="29" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+    </row>
+    <row r="30" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="15"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+    </row>
+    <row r="31" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="15"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+    </row>
+    <row r="32" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="15"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
     </row>
     <row r="33" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="16"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15"/>
+      <c r="A33" s="15"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
     </row>
     <row r="34" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="16"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
+      <c r="A34" s="15"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
     </row>
     <row r="35" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="16"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
+      <c r="A35" s="15"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
     </row>
     <row r="36" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="16"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
     </row>
     <row r="37" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="1"/>

</xml_diff>

<commit_message>
update dropdown surveyJS by text
</commit_message>
<xml_diff>
--- a/datasehat.xlsx
+++ b/datasehat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Documents\sehatselenium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52E0EDC7-1D0E-4DCA-8A4E-8BA82CB610AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E103D934-F274-478D-954B-B28CB9E73765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8604" yWindow="3360" windowWidth="14436" windowHeight="8880" xr2:uid="{204D681D-D5A1-4808-BEE3-E0115C09E5E0}"/>
+    <workbookView xWindow="8280" yWindow="2232" windowWidth="14436" windowHeight="8880" xr2:uid="{204D681D-D5A1-4808-BEE3-E0115C09E5E0}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>nama</t>
   </si>
@@ -106,13 +106,7 @@
     <t>alamat</t>
   </si>
   <si>
-    <t>RIYAN ADRIAN WIBISONO</t>
-  </si>
-  <si>
-    <t>MAKSUDI</t>
-  </si>
-  <si>
-    <t>TIYA SETIYA</t>
+    <t>SIGIT PRATAMA</t>
   </si>
 </sst>
 </file>
@@ -317,9 +311,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -334,6 +325,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -679,156 +673,107 @@
       </c>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" spans="1:8" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="19">
-        <v>110</v>
-      </c>
-      <c r="C2" s="20">
-        <v>70</v>
-      </c>
-      <c r="D2" s="20">
+      <c r="B2" s="18">
+        <v>130</v>
+      </c>
+      <c r="C2" s="19">
+        <v>90</v>
+      </c>
+      <c r="D2" s="19">
         <v>160</v>
       </c>
-      <c r="E2" s="20">
-        <v>62</v>
-      </c>
-      <c r="F2" s="20">
-        <v>80</v>
-      </c>
-      <c r="G2" s="20">
+      <c r="E2" s="19">
+        <v>55</v>
+      </c>
+      <c r="F2" s="19">
         <v>82</v>
       </c>
+      <c r="G2" s="19">
+        <v>85</v>
+      </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="21">
-        <v>120</v>
-      </c>
-      <c r="C3" s="22">
-        <v>80</v>
-      </c>
-      <c r="D3" s="22">
-        <v>160</v>
-      </c>
-      <c r="E3" s="22">
-        <v>60</v>
-      </c>
-      <c r="F3" s="22">
-        <v>84</v>
-      </c>
-      <c r="G3" s="22">
-        <v>84</v>
-      </c>
+      <c r="A3" s="16"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="21">
-        <v>110</v>
-      </c>
-      <c r="C4" s="22">
-        <v>70</v>
-      </c>
-      <c r="D4" s="22">
-        <v>158</v>
-      </c>
-      <c r="E4" s="22">
-        <v>56</v>
-      </c>
-      <c r="F4" s="22">
-        <v>80</v>
-      </c>
-      <c r="G4" s="22">
-        <v>86</v>
-      </c>
+      <c r="A4" s="22"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
+      <c r="A11" s="22"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -872,7 +817,7 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
-      <c r="H17" s="18"/>
+      <c r="H17" s="17"/>
     </row>
     <row r="18" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11"/>
@@ -882,7 +827,7 @@
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
-      <c r="H18" s="18"/>
+      <c r="H18" s="17"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="15"/>

</xml_diff>